<commit_message>
Latest Update for 19 August 2025
</commit_message>
<xml_diff>
--- a/Data/Withdrawal.xlsx
+++ b/Data/Withdrawal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eclipse\Desktop\Automation-Testing-2025\Eclipse\Automation\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abhishekyt\git\repository\Automation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F361EADE-F990-4A38-A185-164B24B4274A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A995C66-2F31-4E26-A786-1879B864DD9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19800" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
   <si>
     <t>Withdrawal_Request_No</t>
   </si>
@@ -424,7 +424,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" bestFit="1" customWidth="1"/>
@@ -594,6 +594,29 @@
         <v>100</v>
       </c>
     </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="4">
+        <v>90904321</v>
+      </c>
+      <c r="B8" s="1">
+        <v>1000421</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="5">
+        <v>100673000000011</v>
+      </c>
+      <c r="F8" s="7">
+        <v>110001023651</v>
+      </c>
+      <c r="G8" s="4">
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>